<commit_message>
Added final changes according to Product Owner feedback
</commit_message>
<xml_diff>
--- a/docs/burndown_charts/BurndownChart sprint 2.xlsx
+++ b/docs/burndown_charts/BurndownChart sprint 2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krzys\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krzys\Desktop\pb docu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD19E726-788D-475C-BDF2-B84629CB2A24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CF5036D-337A-411D-811F-D84D3EC900BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Burndown" sheetId="1" r:id="rId1"/>
@@ -59,9 +59,6 @@
     <t>Story Points</t>
   </si>
   <si>
-    <t>Setup CI with GitHub Actions</t>
-  </si>
-  <si>
     <t>Total</t>
   </si>
   <si>
@@ -69,6 +66,9 @@
   </si>
   <si>
     <t>Bug Fixes</t>
+  </si>
+  <si>
+    <t>Create documentation</t>
   </si>
 </sst>
 </file>
@@ -1124,7 +1124,7 @@
         <v>10</v>
       </c>
       <c r="R3" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S3" s="3">
         <v>5</v>
@@ -1148,7 +1148,7 @@
         <v>5</v>
       </c>
       <c r="R4" s="7" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S4" s="3">
         <v>3</v>
@@ -1172,7 +1172,7 @@
         <v>5</v>
       </c>
       <c r="R5" s="10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="S5" s="11">
         <v>5</v>
@@ -1196,7 +1196,7 @@
         <v>3</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S6" s="8">
         <f>SUM(S3:S5)</f>

</xml_diff>